<commit_message>
Update to Geogame92 + GeogameWeb7
- Geogame92 / GeogameWeb7: fix the freeze (web) / crash (desktop) after
  placing a pipe on a splitting pipe's outlet, and pipes routed downward
  joining the main line's pipe section.
- Pipe costs come from geodata.xlsx instead of fixed 50/60/100; the web
  data (geodata.json) is exported from the same Excel file.
- Username is remembered permanently (desktop file / browser storage).
- Drawdown warning text: QΣ "more than" Qtot_head.
- High scores reset to 0 and bundled solution images removed.
- GeogameWeb6: numpy-array fix and rebuilt web build (from Oct 7).
- Tutorial pictures renamed .PNG -> .png (Linux is case-sensitive).
- requirements.txt for running on Linux (pygame-ce, Python 3.14).
</commit_message>
<xml_diff>
--- a/GeogameUpdater/Currentmodels/GeogameTrainingProgramming/GameAssets/geodata.xlsx
+++ b/GeogameUpdater/Currentmodels/GeogameTrainingProgramming/GameAssets/geodata.xlsx
@@ -2514,7 +2514,7 @@
         </is>
       </c>
       <c r="AW2" s="9" t="n">
-        <v>4010</v>
+        <v>0</v>
       </c>
       <c r="AX2" s="9" t="n">
         <v>0.1</v>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="AW3" t="n">
-        <v>3740</v>
+        <v>0</v>
       </c>
       <c r="AX3" t="n">
         <v>0.1</v>
@@ -2836,7 +2836,7 @@
         </is>
       </c>
       <c r="AW4" s="10" t="n">
-        <v>3610</v>
+        <v>0</v>
       </c>
       <c r="AX4" s="10" t="n">
         <v>0.1</v>
@@ -2997,7 +2997,7 @@
         </is>
       </c>
       <c r="AW5" t="n">
-        <v>3720</v>
+        <v>0</v>
       </c>
       <c r="AX5" t="n">
         <v>0.1</v>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="AW6" s="11" t="n">
-        <v>2970</v>
+        <v>0</v>
       </c>
       <c r="AX6" s="11" t="n">
         <v>0.1</v>
@@ -3319,7 +3319,7 @@
         </is>
       </c>
       <c r="AW7" t="n">
-        <v>3140</v>
+        <v>0</v>
       </c>
       <c r="AX7" t="n">
         <v>0.1</v>
@@ -4124,7 +4124,7 @@
         </is>
       </c>
       <c r="AW12" s="13" t="n">
-        <v>3190</v>
+        <v>0</v>
       </c>
       <c r="AX12" s="13" t="n">
         <v>0.1</v>

</xml_diff>